<commit_message>
content+app: la reflexologie de Guide-moi et du Coucher passe par un lien
Les gestes doux n'inventent plus de sequence de reflexologie : quand un
protocole valide couvre le mois, le texte renvoie vers lui et le bloc porte
un bouton « Ouvrir la sequence ». 136 liens dans Guide-moi, 23 dans le
Coucher (M1 a M23), tous verifies : protocole publie, bornes d'age du mois
respectees, titre exact. Les etapes inventees du Coucher sont retirees.

Titres des gestes doux : plus de prefixe « Geste doux », la precision seule.
Skills mis a jour en consequence.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GUIDE2_situations.xlsx
+++ b/GUIDE2_situations.xlsx
@@ -17762,7 +17762,7 @@
       </c>
       <c r="G326" s="41" t="inlineStr">
         <is>
-          <t>Se déplacer assis est une variante normale du développement : ni à corriger, ni à empêcher, ni à rééduquer.</t>
+          <t>Signal fréquent d'un enfant installé assis trop tôt : lui rendre du temps au sol et les passages entre positions, par le jeu, et en parler au suivi.</t>
         </is>
       </c>
       <c r="H326" s="39" t="inlineStr">
@@ -23484,17 +23484,17 @@
       </c>
       <c r="E438" s="41" t="inlineStr">
         <is>
-          <t>La comparaison des jalons</t>
+          <t>La comparaison des étapes</t>
         </is>
       </c>
       <c r="F438" s="41" t="inlineStr">
         <is>
-          <t>Les autres marchent déjà</t>
+          <t>J'ai peur qu'il soit en retard</t>
         </is>
       </c>
       <c r="G438" s="41" t="inlineStr">
         <is>
-          <t>Désamorcer la comparaison des jalons au moment précis où les écarts entre enfants sont les plus visibles.</t>
+          <t>Désamorcer la comparaison des étapes (marche, langage, repas, contacts) et la pression qu'elle fait peser sur l'enfant, au moment où les écarts sont les plus visibles.</t>
         </is>
       </c>
       <c r="H438" s="39" t="inlineStr">
@@ -23509,7 +23509,7 @@
       </c>
       <c r="J438" s="41" t="inlineStr">
         <is>
-          <t>La comparaison des jalons / Les autres marchent déjà</t>
+          <t>La comparaison des étapes / J'ai peur qu'il soit en retard</t>
         </is>
       </c>
       <c r="K438" s="41" t="inlineStr">
@@ -43647,7 +43647,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="32">
       <c r="A4" s="52" t="inlineStr">
         <is>
@@ -43725,7 +43724,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="32">
       <c r="A13" s="52" t="inlineStr">
         <is>
@@ -43813,7 +43811,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="32">
       <c r="A23" s="52" t="inlineStr">
         <is>
@@ -43911,7 +43908,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="32">
       <c r="A34" s="52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
content(guide): situations recentes publiees (M3, M5-M9, M11-M15, M18, M21, M23)
- M11 Pleurs : « Les hurlements du refus / Il s'affirme en criant » remplace « L'opposition qui arrive »
- Molaires deplacees de M11/M12 vers M15 (nouvelle carte Dents)
- Nouvelle carte Colere & emotions en M14 et M18
- Corrections de textes sur les autres mois ; tableau GUIDE2_situations.xlsx a jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GUIDE2_situations.xlsx
+++ b/GUIDE2_situations.xlsx
@@ -1057,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K856"/>
+  <dimension ref="A1:K857"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="31" min="1" max="1"/>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="C26" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D26" s="39" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="C27" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D27" s="39" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="C28" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D28" s="39" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D29" s="39" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D30" s="39" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="C31" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D31" s="39" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="C59" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D59" s="39" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="C60" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D60" s="39" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="C61" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D61" s="39" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="C62" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D62" s="39" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="C63" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D63" s="39" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="C64" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D64" s="39" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="C93" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D93" s="39" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="C94" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D94" s="39" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="C95" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D95" s="39" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="C96" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D96" s="39" t="inlineStr">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C97" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D97" s="39" t="inlineStr">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="C98" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D98" s="39" t="inlineStr">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="C127" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D127" s="39" t="inlineStr">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="C128" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D128" s="39" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="C129" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D129" s="39" t="inlineStr">
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C130" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D130" s="39" t="inlineStr">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="C131" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D131" s="39" t="inlineStr">
@@ -7805,7 +7805,7 @@
       </c>
       <c r="C132" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D132" s="39" t="inlineStr">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="C161" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D161" s="39" t="inlineStr">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="C162" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D162" s="39" t="inlineStr">
@@ -9394,7 +9394,7 @@
       </c>
       <c r="C163" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D163" s="39" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="C164" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D164" s="39" t="inlineStr">
@@ -9496,7 +9496,7 @@
       </c>
       <c r="C165" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D165" s="39" t="inlineStr">
@@ -9547,7 +9547,7 @@
       </c>
       <c r="C166" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D166" s="39" t="inlineStr">
@@ -11006,7 +11006,7 @@
       </c>
       <c r="C194" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D194" s="39" t="inlineStr">
@@ -11057,7 +11057,7 @@
       </c>
       <c r="C195" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D195" s="39" t="inlineStr">
@@ -11108,7 +11108,7 @@
       </c>
       <c r="C196" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D196" s="39" t="inlineStr">
@@ -11159,7 +11159,7 @@
       </c>
       <c r="C197" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D197" s="39" t="inlineStr">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="C198" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D198" s="39" t="inlineStr">
@@ -11261,7 +11261,7 @@
       </c>
       <c r="C199" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D199" s="39" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="C225" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D225" s="39" t="inlineStr">
@@ -12634,7 +12634,7 @@
       </c>
       <c r="C226" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D226" s="39" t="inlineStr">
@@ -12685,7 +12685,7 @@
       </c>
       <c r="C227" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D227" s="39" t="inlineStr">
@@ -12736,7 +12736,7 @@
       </c>
       <c r="C228" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D228" s="39" t="inlineStr">
@@ -14341,7 +14341,7 @@
       </c>
       <c r="C259" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D259" s="39" t="inlineStr">
@@ -14392,7 +14392,7 @@
       </c>
       <c r="C260" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D260" s="39" t="inlineStr">
@@ -14431,7 +14431,7 @@
       </c>
       <c r="C261" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D261" s="39" t="inlineStr">
@@ -14482,7 +14482,7 @@
       </c>
       <c r="C262" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D262" s="39" t="inlineStr">
@@ -16161,7 +16161,7 @@
       </c>
       <c r="C295" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D295" s="39" t="inlineStr">
@@ -16212,7 +16212,7 @@
       </c>
       <c r="C296" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D296" s="39" t="inlineStr">
@@ -16263,7 +16263,7 @@
       </c>
       <c r="C297" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D297" s="39" t="inlineStr">
@@ -16314,7 +16314,7 @@
       </c>
       <c r="C298" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D298" s="39" t="inlineStr">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="C332" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D332" s="39" t="inlineStr">
@@ -18111,7 +18111,7 @@
       </c>
       <c r="C333" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D333" s="39" t="inlineStr">
@@ -18162,7 +18162,7 @@
       </c>
       <c r="C334" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D334" s="39" t="inlineStr">
@@ -18213,7 +18213,7 @@
       </c>
       <c r="C335" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D335" s="39" t="inlineStr">
@@ -19939,7 +19939,7 @@
       </c>
       <c r="C369" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D369" s="39" t="inlineStr">
@@ -19990,7 +19990,7 @@
       </c>
       <c r="C370" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D370" s="39" t="inlineStr">
@@ -20041,7 +20041,7 @@
       </c>
       <c r="C371" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D371" s="39" t="inlineStr">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="C372" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D372" s="39" t="inlineStr">
@@ -21740,7 +21740,7 @@
       </c>
       <c r="C404" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D404" s="39" t="inlineStr">
@@ -21791,7 +21791,7 @@
       </c>
       <c r="C405" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D405" s="39" t="inlineStr">
@@ -21842,7 +21842,7 @@
       </c>
       <c r="C406" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D406" s="39" t="inlineStr">
@@ -21893,7 +21893,7 @@
       </c>
       <c r="C407" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D407" s="39" t="inlineStr">
@@ -23529,7 +23529,7 @@
       </c>
       <c r="C439" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D439" s="39" t="inlineStr">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="C440" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D440" s="39" t="inlineStr">
@@ -23631,7 +23631,7 @@
       </c>
       <c r="C441" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D441" s="39" t="inlineStr">
@@ -23682,7 +23682,7 @@
       </c>
       <c r="C442" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D442" s="39" t="inlineStr">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="C475" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D475" s="39" t="inlineStr">
@@ -25364,7 +25364,7 @@
       </c>
       <c r="C476" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D476" s="39" t="inlineStr">
@@ -25411,7 +25411,7 @@
       </c>
       <c r="C477" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D477" s="39" t="inlineStr">
@@ -25458,7 +25458,7 @@
       </c>
       <c r="C478" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D478" s="39" t="inlineStr">
@@ -27100,7 +27100,7 @@
       </c>
       <c r="C512" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D512" s="39" t="inlineStr">
@@ -27147,7 +27147,7 @@
       </c>
       <c r="C513" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D513" s="39" t="inlineStr">
@@ -27194,7 +27194,7 @@
       </c>
       <c r="C514" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D514" s="39" t="inlineStr">
@@ -27241,7 +27241,7 @@
       </c>
       <c r="C515" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D515" s="39" t="inlineStr">
@@ -27288,7 +27288,7 @@
       </c>
       <c r="C516" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D516" s="39" t="inlineStr">
@@ -28812,7 +28812,7 @@
       </c>
       <c r="C548" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D548" s="39" t="inlineStr">
@@ -28859,7 +28859,7 @@
       </c>
       <c r="C549" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D549" s="39" t="inlineStr">
@@ -28906,7 +28906,7 @@
       </c>
       <c r="C550" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D550" s="39" t="inlineStr">
@@ -28953,7 +28953,7 @@
       </c>
       <c r="C551" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D551" s="39" t="inlineStr">
@@ -30399,7 +30399,7 @@
       </c>
       <c r="C581" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D581" s="39" t="inlineStr">
@@ -30446,7 +30446,7 @@
       </c>
       <c r="C582" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D582" s="39" t="inlineStr">
@@ -30493,7 +30493,7 @@
       </c>
       <c r="C583" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D583" s="39" t="inlineStr">
@@ -30540,7 +30540,7 @@
       </c>
       <c r="C584" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D584" s="39" t="inlineStr">
@@ -32017,7 +32017,7 @@
       </c>
       <c r="C615" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D615" s="39" t="inlineStr">
@@ -32064,7 +32064,7 @@
       </c>
       <c r="C616" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D616" s="39" t="inlineStr">
@@ -32111,7 +32111,7 @@
       </c>
       <c r="C617" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D617" s="39" t="inlineStr">
@@ -32158,7 +32158,7 @@
       </c>
       <c r="C618" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D618" s="39" t="inlineStr">
@@ -33345,12 +33345,12 @@
       </c>
       <c r="C643" s="42" t="inlineStr">
         <is>
-          <t>Motricité &amp; exploration</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D643" s="39" t="inlineStr">
         <is>
-          <t>Motricité &amp; exploration</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="E643" s="41" t="inlineStr">
@@ -33369,7 +33369,11 @@
           <t>à écrire</t>
         </is>
       </c>
-      <c r="I643" s="41" t="n"/>
+      <c r="I643" s="41" t="inlineStr">
+        <is>
+          <t>Thème changé le 28/09/2026 : refus d'un soin fait par l'adulte, la mère le cherche dans la colère, pas dans la motricité.</t>
+        </is>
+      </c>
       <c r="J643" s="41" t="n"/>
       <c r="K643" s="41" t="n"/>
     </row>
@@ -33584,7 +33588,7 @@
       </c>
       <c r="C648" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D648" s="39" t="inlineStr">
@@ -33631,7 +33635,7 @@
       </c>
       <c r="C649" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D649" s="39" t="inlineStr">
@@ -33678,7 +33682,7 @@
       </c>
       <c r="C650" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D650" s="39" t="inlineStr">
@@ -33725,7 +33729,7 @@
       </c>
       <c r="C651" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D651" s="39" t="inlineStr">
@@ -33772,7 +33776,7 @@
       </c>
       <c r="C652" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D652" s="39" t="inlineStr">
@@ -33819,7 +33823,7 @@
       </c>
       <c r="C653" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D653" s="39" t="inlineStr">
@@ -34979,12 +34983,12 @@
       </c>
       <c r="C677" s="42" t="inlineStr">
         <is>
-          <t>Motricité &amp; exploration</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D677" s="39" t="inlineStr">
         <is>
-          <t>Motricité &amp; exploration</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="E677" s="41" t="inlineStr">
@@ -35007,7 +35011,11 @@
           <t>à écrire</t>
         </is>
       </c>
-      <c r="I677" s="41" t="n"/>
+      <c r="I677" s="41" t="inlineStr">
+        <is>
+          <t>Thème changé le 28/09/2026 : refus d'un soin fait par l'adulte, la mère le cherche dans la colère, pas dans la motricité.</t>
+        </is>
+      </c>
       <c r="J677" s="41" t="n"/>
       <c r="K677" s="41" t="inlineStr">
         <is>
@@ -35351,7 +35359,7 @@
       </c>
       <c r="C685" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D685" s="39" t="inlineStr">
@@ -35398,7 +35406,7 @@
       </c>
       <c r="C686" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D686" s="39" t="inlineStr">
@@ -35445,7 +35453,7 @@
       </c>
       <c r="C687" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D687" s="39" t="inlineStr">
@@ -35492,7 +35500,7 @@
       </c>
       <c r="C688" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D688" s="39" t="inlineStr">
@@ -35539,7 +35547,7 @@
       </c>
       <c r="C689" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D689" s="39" t="inlineStr">
@@ -35586,7 +35594,7 @@
       </c>
       <c r="C690" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D690" s="39" t="inlineStr">
@@ -36899,7 +36907,11 @@
           <t>à écrire</t>
         </is>
       </c>
-      <c r="I717" s="41" t="n"/>
+      <c r="I717" s="41" t="inlineStr">
+        <is>
+          <t>Ligne libérée le 28/09/2026 : doublon du siège auto de M18, à redéfinir lors de la passe Motricité du mois.</t>
+        </is>
+      </c>
       <c r="J717" s="41" t="n"/>
       <c r="K717" s="41" t="n"/>
     </row>
@@ -37114,7 +37126,7 @@
       </c>
       <c r="C722" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D722" s="39" t="inlineStr">
@@ -37161,7 +37173,7 @@
       </c>
       <c r="C723" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D723" s="39" t="inlineStr">
@@ -37208,7 +37220,7 @@
       </c>
       <c r="C724" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D724" s="39" t="inlineStr">
@@ -37255,7 +37267,7 @@
       </c>
       <c r="C725" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D725" s="39" t="inlineStr">
@@ -37302,7 +37314,7 @@
       </c>
       <c r="C726" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D726" s="39" t="inlineStr">
@@ -37349,7 +37361,7 @@
       </c>
       <c r="C727" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D727" s="39" t="inlineStr">
@@ -38889,7 +38901,7 @@
       </c>
       <c r="C759" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D759" s="39" t="inlineStr">
@@ -38936,7 +38948,7 @@
       </c>
       <c r="C760" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D760" s="39" t="inlineStr">
@@ -38983,7 +38995,7 @@
       </c>
       <c r="C761" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D761" s="39" t="inlineStr">
@@ -39030,7 +39042,7 @@
       </c>
       <c r="C762" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D762" s="39" t="inlineStr">
@@ -39077,7 +39089,7 @@
       </c>
       <c r="C763" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D763" s="39" t="inlineStr">
@@ -39124,7 +39136,7 @@
       </c>
       <c r="C764" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D764" s="39" t="inlineStr">
@@ -40268,12 +40280,12 @@
       </c>
       <c r="C788" s="42" t="inlineStr">
         <is>
-          <t>Motricité &amp; exploration</t>
+          <t>Autonomie &amp; propreté</t>
         </is>
       </c>
       <c r="D788" s="39" t="inlineStr">
         <is>
-          <t>Motricité &amp; exploration</t>
+          <t>Autonomie &amp; propreté</t>
         </is>
       </c>
       <c r="E788" s="41" t="inlineStr">
@@ -40296,7 +40308,11 @@
           <t>à écrire</t>
         </is>
       </c>
-      <c r="I788" s="41" t="n"/>
+      <c r="I788" s="41" t="inlineStr">
+        <is>
+          <t>Thème changé le 28/09/2026 : découverte du corps pendant le change, ni refus ni « faire seul » — rangé avec la propreté.</t>
+        </is>
+      </c>
       <c r="J788" s="41" t="n"/>
       <c r="K788" s="41" t="inlineStr">
         <is>
@@ -40656,7 +40672,7 @@
       </c>
       <c r="C796" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D796" s="39" t="inlineStr">
@@ -40703,7 +40719,7 @@
       </c>
       <c r="C797" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D797" s="39" t="inlineStr">
@@ -40750,7 +40766,7 @@
       </c>
       <c r="C798" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D798" s="39" t="inlineStr">
@@ -40797,7 +40813,7 @@
       </c>
       <c r="C799" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D799" s="39" t="inlineStr">
@@ -40844,7 +40860,7 @@
       </c>
       <c r="C800" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D800" s="39" t="inlineStr">
@@ -40891,7 +40907,7 @@
       </c>
       <c r="C801" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D801" s="39" t="inlineStr">
@@ -42459,7 +42475,7 @@
       </c>
       <c r="C833" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D833" s="39" t="inlineStr">
@@ -42510,7 +42526,7 @@
       </c>
       <c r="C834" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D834" s="39" t="inlineStr">
@@ -42561,7 +42577,7 @@
       </c>
       <c r="C835" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D835" s="39" t="inlineStr">
@@ -42612,7 +42628,7 @@
       </c>
       <c r="C836" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D836" s="39" t="inlineStr">
@@ -42663,7 +42679,7 @@
       </c>
       <c r="C837" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D837" s="39" t="inlineStr">
@@ -42710,7 +42726,7 @@
       </c>
       <c r="C838" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D838" s="39" t="inlineStr">
@@ -42757,7 +42773,7 @@
       </c>
       <c r="C839" s="47" t="inlineStr">
         <is>
-          <t>Pleurs, colère et débordement</t>
+          <t>Pleurs &amp; colère</t>
         </is>
       </c>
       <c r="D839" s="39" t="inlineStr">
@@ -43609,6 +43625,56 @@
       <c r="I856" s="31" t="inlineStr">
         <is>
           <t>Créée le 01/09/2026. La diarrhée était absente des 855 situations sur 24 mois. Place libérée par le passage du haut-le-cœur à la cuillère en Alimentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="B857" s="31" t="inlineStr">
+        <is>
+          <t>M12-M17 · Marche</t>
+        </is>
+      </c>
+      <c r="C857" s="31" t="inlineStr">
+        <is>
+          <t>Alimentation</t>
+        </is>
+      </c>
+      <c r="D857" s="31" t="inlineStr">
+        <is>
+          <t>Alimentation</t>
+        </is>
+      </c>
+      <c r="E857" s="31" t="inlineStr">
+        <is>
+          <t>L'allaitement après un an</t>
+        </is>
+      </c>
+      <c r="F857" s="31" t="inlineStr">
+        <is>
+          <t>je continue et ça dérange</t>
+        </is>
+      </c>
+      <c r="G857" s="31" t="inlineStr">
+        <is>
+          <t>Aider la mère à expliquer son choix en une phrase et à le garder : pas de date d'arrêt en France, l'OMS cite deux ans et au-delà comme repère. Protéger les tétées qui comptent plutôt que se justifier.</t>
+        </is>
+      </c>
+      <c r="H857" s="31" t="inlineStr">
+        <is>
+          <t>écrit</t>
+        </is>
+      </c>
+      <c r="I857" s="31" t="inlineStr">
+        <is>
+          <t>Situation créée le 28/09/2026 : M11 traite le sevrage sous quatre angles, rien ne traitait la mère qui poursuit.</t>
+        </is>
+      </c>
+      <c r="J857" s="31" t="inlineStr">
+        <is>
+          <t>L'allaitement après un an / je continue et ça dérange</t>
         </is>
       </c>
     </row>

</xml_diff>